<commit_message>
Dashboard update 2026-08-10 14:17
</commit_message>
<xml_diff>
--- a/excel/Nordstreet.xlsx
+++ b/excel/Nordstreet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Investavimas 2026.06.03\Nordstreet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.08.08\Nordstreet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C49BCC-641F-40CF-8CCC-CC4EBED43235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41C2263E-0998-47DB-BB8D-5B72A05A20BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Apžvalga" sheetId="1" r:id="rId1"/>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="R3" s="5">
         <f>U3-P3</f>
-        <v>91.860000000000127</v>
+        <v>93.220000000000027</v>
       </c>
       <c r="S3" s="5">
         <f>SUM(L3:L200)</f>
@@ -3516,23 +3516,23 @@
       </c>
       <c r="T3" s="5">
         <f>SUM(M3:M200)</f>
-        <v>116.21</v>
+        <v>117.57</v>
       </c>
       <c r="U3" s="5">
         <f>O3+T3+Q3</f>
-        <v>1115.1500000000001</v>
+        <v>1116.51</v>
       </c>
       <c r="V3" s="5">
         <f>U3-O3</f>
-        <v>165.15000000000009</v>
+        <v>166.51</v>
       </c>
       <c r="W3" s="15">
         <f>(U3-O3)/O3</f>
-        <v>0.17384210526315799</v>
+        <v>0.1752736842105263</v>
       </c>
       <c r="X3" s="15">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>0.15337591767311098</v>
+        <v>0.15263281464576722</v>
       </c>
       <c r="AC3" s="5" t="str">
         <f ca="1">'Mesiheina tee 5 ir 8 (1)'!AA2</f>
@@ -3577,11 +3577,11 @@
       </c>
       <c r="J4" s="9">
         <f ca="1">'Bistryčios g. 27 (3)'!B13</f>
-        <v>-26</v>
+        <v>-31</v>
       </c>
       <c r="K4" s="9">
         <f ca="1">'Bistryčios g. 27 (3)'!S3</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="L4" s="5">
         <f>'Bistryčios g. 27 (3)'!N3</f>
@@ -3634,11 +3634,11 @@
       </c>
       <c r="J5" s="9">
         <f ca="1">'2 MW saulės elektrinių par. (9)'!B13</f>
-        <v>-211</v>
+        <v>-216</v>
       </c>
       <c r="K5" s="9">
         <f ca="1">'2 MW saulės elektrinių par. (9)'!S3</f>
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="L5" s="5">
         <f>'2 MW saulės elektrinių par. (9)'!N3</f>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="J6" s="9">
         <f ca="1">'Kvartalas "Asiūklės parkas” (2)'!B13</f>
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="K6" s="9" t="str">
         <f ca="1">'Kvartalas "Asiūklės parkas” (2)'!S3</f>
@@ -3976,11 +3976,11 @@
       </c>
       <c r="J11" s="9">
         <f ca="1">'Vidiškių vs., Žemaitkiemio (2)'!B13</f>
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="K11" s="9">
         <f ca="1">'Vidiškių vs., Žemaitkiemio (2)'!S3</f>
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="L11" s="5">
         <f>'Vidiškių vs., Žemaitkiemio (2)'!N3</f>
@@ -4090,11 +4090,11 @@
       </c>
       <c r="J13" s="9">
         <f ca="1">'Vilniaus g. 38 38A 38B (1)'!B13</f>
-        <v>-32</v>
+        <v>-37</v>
       </c>
       <c r="K13" s="9">
         <f ca="1">'Vilniaus g. 38 38A 38B (1)'!S3</f>
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="L13" s="5">
         <f>'Vilniaus g. 38 38A 38B (1)'!N3</f>
@@ -4204,7 +4204,7 @@
       </c>
       <c r="J15" s="9">
         <f ca="1">'Viensėdžio g. 36A (3)'!B13</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="K15" s="9" t="str">
         <f ca="1">'Viensėdžio g. 36A (3)'!S3</f>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="J16" s="9">
         <f ca="1">'Šaltinio g. 7, Panevėžys (1)'!B13</f>
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="K16" s="9" t="str">
         <f ca="1">'Šaltinio g. 7, Panevėžys (1)'!S3</f>
@@ -4318,11 +4318,11 @@
       </c>
       <c r="J17" s="9">
         <f ca="1">'Mozūriškių g. 17 - 3, Vilnius'!B13</f>
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="K17" s="9">
         <f ca="1">'Mozūriškių g. 17 - 3, Vilnius'!S3</f>
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="L17" s="5">
         <f>'Mozūriškių g. 17 - 3, Vilnius'!N3</f>
@@ -4375,11 +4375,11 @@
       </c>
       <c r="J18" s="9">
         <f ca="1">'Parko g. 21 Pergalės g. 36A (1)'!B13</f>
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="K18" s="9">
         <f ca="1">'Parko g. 21 Pergalės g. 36A (1)'!S3</f>
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="L18" s="5">
         <f>'Parko g. 21 Pergalės g. 36A (1)'!N3</f>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="J20" s="9">
         <f ca="1">'Baltų Avenue (1)'!B13</f>
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="K20" s="9" t="str">
         <f ca="1">'Baltų Avenue (1)'!S3</f>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="J21" s="9">
         <f ca="1">'"Filleo Home", Palanga (3)'!B13</f>
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="K21" s="9" t="str">
         <f ca="1">'"Filleo Home", Palanga (3)'!S3</f>
@@ -4603,11 +4603,11 @@
       </c>
       <c r="J22" s="9">
         <f ca="1">'Sklypų masyvas Loo, Parnu (1)'!B13</f>
-        <v>208</v>
-      </c>
-      <c r="K22" s="9" t="str">
+        <v>203</v>
+      </c>
+      <c r="K22" s="9">
         <f ca="1">'Sklypų masyvas Loo, Parnu (1)'!S3</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="L22" s="5">
         <f>'Sklypų masyvas Loo, Parnu (1)'!N3</f>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="AC22" s="5" t="str">
         <f ca="1">'Sklypų masyvas Loo, Parnu (1)'!AA2</f>
-        <v/>
+        <v>+</v>
       </c>
     </row>
     <row r="23" spans="1:29" x14ac:dyDescent="0.25">
@@ -4660,11 +4660,11 @@
       </c>
       <c r="J23" s="9">
         <f ca="1">'Liepų g. 3, Vyšniūnai (1)'!B13</f>
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="K23" s="9">
         <f ca="1">'Liepų g. 3, Vyšniūnai (1)'!S3</f>
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="L23" s="5">
         <f>'Liepų g. 3, Vyšniūnai (1)'!N3</f>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="J24" s="9">
         <f ca="1">'Basliupio g. 14, Panevėžys (3)'!B13</f>
-        <v>557</v>
+        <v>552</v>
       </c>
       <c r="K24" s="9" t="str">
         <f ca="1">'Basliupio g. 14, Panevėžys (3)'!S3</f>
@@ -4729,7 +4729,7 @@
       </c>
       <c r="M24" s="5">
         <f>'Basliupio g. 14, Panevėžys (3)'!P3</f>
-        <v>2.36</v>
+        <v>2.96</v>
       </c>
       <c r="AC24" s="5" t="str">
         <f ca="1">'Basliupio g. 14, Panevėžys (3)'!AA2</f>
@@ -4774,7 +4774,7 @@
       </c>
       <c r="J25" s="9">
         <f ca="1">'Mėguvos g. 6 ir 8, Palanga (2)'!B13</f>
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="K25" s="9" t="str">
         <f ca="1">'Mėguvos g. 6 ir 8, Palanga (2)'!S3</f>
@@ -4831,7 +4831,7 @@
       </c>
       <c r="J26" s="9">
         <f ca="1">'"Filleo Home", Palanga (10)'!B13</f>
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="K26" s="9" t="str">
         <f ca="1">'"Filleo Home", Palanga (10)'!S3</f>
@@ -4843,7 +4843,7 @@
       </c>
       <c r="M26" s="5">
         <f>'"Filleo Home", Palanga (10)'!P3</f>
-        <v>1.49</v>
+        <v>2.25</v>
       </c>
       <c r="AC26" s="5" t="str">
         <f ca="1">'"Filleo Home", Palanga (10)'!AA2</f>
@@ -4888,7 +4888,7 @@
       </c>
       <c r="J27" s="9">
         <f ca="1">'Baltų Avenue (11)'!B13</f>
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="K27" s="9" t="str">
         <f ca="1">'Baltų Avenue (11)'!S3</f>
@@ -4945,7 +4945,7 @@
       </c>
       <c r="J28" s="9">
         <f ca="1">'Plento g. 5A, Trakai (2)'!B13</f>
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="K28" s="9" t="str">
         <f ca="1">'Plento g. 5A, Trakai (2)'!S3</f>
@@ -5573,7 +5573,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D13" s="8">
         <v>46371</v>
@@ -6837,7 +6837,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="D13" s="8">
         <v>46345</v>
@@ -9136,7 +9136,7 @@
       </c>
       <c r="S3" s="3">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
@@ -9483,7 +9483,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D13" s="8">
         <v>46323</v>
@@ -10379,7 +10379,7 @@
       </c>
       <c r="S3" s="3">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
@@ -10758,7 +10758,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D13" s="8">
         <v>46284</v>
@@ -12040,7 +12040,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>399</v>
+        <v>394</v>
       </c>
       <c r="D13" s="8">
         <v>46273</v>
@@ -12808,9 +12808,6 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FFFFC000"/>
-  </sheetPr>
   <dimension ref="A1:AA42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -13398,7 +13395,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D13" s="8">
         <v>46248</v>
@@ -15491,7 +15488,7 @@
       </c>
       <c r="S3" s="3">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
@@ -15872,7 +15869,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>-32</v>
+        <v>-37</v>
       </c>
       <c r="D13" s="8">
         <v>46207</v>
@@ -17983,7 +17980,7 @@
       </c>
       <c r="L1" s="15">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>0.15337591767311098</v>
+        <v>0.15263281464576722</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -19788,14 +19785,14 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="8">
         <f ca="1">TODAY()</f>
-        <v>46239</v>
+        <v>46244</v>
       </c>
       <c r="B200" s="2"/>
       <c r="C200" s="2"/>
       <c r="D200" s="2"/>
       <c r="K200" s="28">
         <f>Apžvalga!U3</f>
-        <v>1115.1500000000001</v>
+        <v>1116.51</v>
       </c>
     </row>
   </sheetData>
@@ -20008,7 +20005,7 @@
       </c>
       <c r="S3" s="3">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
@@ -20389,7 +20386,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="D13" s="8">
         <v>46199</v>
@@ -26882,7 +26879,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="D13" s="8">
         <v>46101</v>
@@ -27904,7 +27901,7 @@
       </c>
       <c r="S3" s="3">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
@@ -28245,7 +28242,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>-211</v>
+        <v>-216</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="5"/>
@@ -29134,7 +29131,7 @@
       </c>
       <c r="S3" s="3">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
@@ -29523,7 +29520,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>-26</v>
+        <v>-31</v>
       </c>
       <c r="D13" s="8">
         <v>46086</v>
@@ -32111,7 +32108,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D13" s="8">
         <v>46561</v>
@@ -33180,7 +33177,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="D13" s="8">
         <v>46515</v>
@@ -34121,7 +34118,7 @@
       </c>
       <c r="P3" s="5">
         <f>H42+I42</f>
-        <v>1.49</v>
+        <v>2.25</v>
       </c>
       <c r="Q3" s="15" t="str">
         <f>IF(M3=N3,XIRR(Z2:Z26,Y2:Y26),"")</f>
@@ -34163,13 +34160,21 @@
       <c r="F4" s="5">
         <v>0.76</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="G4" s="5">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>0.76</v>
+      </c>
+      <c r="I4" s="5">
+        <v>0</v>
+      </c>
+      <c r="J4" s="8">
+        <v>46244</v>
+      </c>
+      <c r="K4" s="9">
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
       <c r="Y4" s="8">
         <f t="shared" ref="Y4:Y41" si="1">J3</f>
@@ -34206,11 +34211,11 @@
       </c>
       <c r="Y5" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46244</v>
       </c>
       <c r="Z5" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
@@ -34432,7 +34437,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="5"/>
@@ -35071,7 +35076,7 @@
       </c>
       <c r="H42" s="5">
         <f t="shared" si="4"/>
-        <v>1.49</v>
+        <v>2.25</v>
       </c>
       <c r="I42" s="5">
         <f t="shared" si="4"/>
@@ -35644,7 +35649,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="D13" s="8">
         <v>46490</v>
@@ -36525,7 +36530,7 @@
       </c>
       <c r="P3" s="5">
         <f>H42+I42</f>
-        <v>2.36</v>
+        <v>2.96</v>
       </c>
       <c r="Q3" s="15" t="str">
         <f>IF(M3=N3,XIRR(Z2:Z26,Y2:Y26),"")</f>
@@ -36649,13 +36654,21 @@
       <c r="F6" s="5">
         <v>0.6</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="G6" s="5">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="I6" s="5">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8">
+        <v>46244</v>
+      </c>
+      <c r="K6" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="Y6" s="8">
         <f t="shared" si="1"/>
@@ -36692,11 +36705,11 @@
       </c>
       <c r="Y7" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46244</v>
       </c>
       <c r="Z7" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
@@ -36870,7 +36883,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>557</v>
+        <v>552</v>
       </c>
       <c r="D13" s="8">
         <v>46455</v>
@@ -37587,7 +37600,7 @@
       </c>
       <c r="H42" s="5">
         <f t="shared" si="4"/>
-        <v>2.36</v>
+        <v>2.96</v>
       </c>
       <c r="I42" s="5">
         <f t="shared" si="4"/>
@@ -37838,7 +37851,7 @@
       </c>
       <c r="S3" s="3">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
@@ -38163,7 +38176,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="D13" s="8">
         <v>46429</v>
@@ -38998,7 +39011,7 @@
       </c>
       <c r="AA2" s="3" t="str">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")&gt;0,"+","")</f>
-        <v/>
+        <v>+</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
@@ -39057,9 +39070,9 @@
         <f>IF(M3=N3,B14,"")</f>
         <v/>
       </c>
-      <c r="S3" s="3" t="str">
+      <c r="S3" s="3">
         <f ca="1">IF(COUNTIFS(D:D,"&lt;"&amp;TODAY(),J:J,"")=0,"",TODAY()-_xlfn.MINIFS(D:D,D:D,"&lt;"&amp;TODAY(),J:J,""))</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
@@ -39408,7 +39421,7 @@
       </c>
       <c r="B13" s="9">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D13" s="8">
         <v>46394</v>

</xml_diff>